<commit_message>
Added script for plot mana values by format. Added slight edits to previous scripts and datasets.
</commit_message>
<xml_diff>
--- a/Data/002_Example_mana_curve_types/002_Example_Distributions_Mana_Curve_Types_2026.xlsx
+++ b/Data/002_Example_mana_curve_types/002_Example_Distributions_Mana_Curve_Types_2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\falkn\Documents\Projects\Magic_Deck_building_Statistics\Data\001_Example_decklist_Hitmonkey\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\falkn\Documents\Projects\Magic_Deck_building_Statistics\Data\002_Example_mana_curve_types\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1CB6B560-5E14-4319-9406-DBF850C56C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E11BFEDD-188D-43D1-8B3B-F0D5B346E82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1EEAAFF7-C7DB-41B1-ACB2-DFA001B71D6B}"/>
   </bookViews>
@@ -899,7 +899,7 @@
         <v>1</v>
       </c>
       <c r="B42">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C42" t="s">
         <v>4</v>
@@ -910,7 +910,7 @@
         <v>2</v>
       </c>
       <c r="B43">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C43" t="s">
         <v>4</v>
@@ -921,7 +921,7 @@
         <v>3</v>
       </c>
       <c r="B44">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C44" t="s">
         <v>4</v>
@@ -932,7 +932,7 @@
         <v>4</v>
       </c>
       <c r="B45">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C45" t="s">
         <v>4</v>
@@ -943,7 +943,7 @@
         <v>5</v>
       </c>
       <c r="B46">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C46" t="s">
         <v>4</v>
@@ -954,7 +954,7 @@
         <v>6</v>
       </c>
       <c r="B47">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C47" t="s">
         <v>4</v>
@@ -976,7 +976,7 @@
         <v>8</v>
       </c>
       <c r="B49">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C49" t="s">
         <v>4</v>
@@ -987,7 +987,7 @@
         <v>9</v>
       </c>
       <c r="B50">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C50" t="s">
         <v>4</v>
@@ -998,7 +998,7 @@
         <v>10</v>
       </c>
       <c r="B51">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C51" t="s">
         <v>4</v>
@@ -1141,7 +1141,7 @@
         <v>3</v>
       </c>
       <c r="B64">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C64" t="s">
         <v>6</v>
@@ -1174,7 +1174,7 @@
         <v>6</v>
       </c>
       <c r="B67">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C67" t="s">
         <v>6</v>
@@ -1185,7 +1185,7 @@
         <v>7</v>
       </c>
       <c r="B68">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C68" t="s">
         <v>6</v>

</xml_diff>